<commit_message>
Checkpoint 15 - Import module validated
</commit_message>
<xml_diff>
--- a/public/SubTracker_Import_Template.xlsx
+++ b/public/SubTracker_Import_Template.xlsx
@@ -463,11 +463,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Company Name</v>
+  <dimension ref="A1:R1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Company Name*</v>
       </c>
       <c r="B1" t="str">
         <v>Trade</v>
@@ -482,21 +482,48 @@
         <v>Phone</v>
       </c>
       <c r="F1" t="str">
+        <v>Address 1</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Address 2</v>
+      </c>
+      <c r="H1" t="str">
+        <v>City</v>
+      </c>
+      <c r="I1" t="str">
+        <v>State</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Zip Code</v>
+      </c>
+      <c r="K1" t="str">
+        <v>NJ PWC #</v>
+      </c>
+      <c r="L1" t="str">
+        <v>NJ BRC #</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Sage ERP ID</v>
+      </c>
+      <c r="N1" t="str">
+        <v>BRC Name Control</v>
+      </c>
+      <c r="O1" t="str">
         <v>Notes</v>
       </c>
-      <c r="G1" t="str">
+      <c r="P1" t="str">
         <v>External ID</v>
       </c>
-      <c r="H1" t="str">
+      <c r="Q1" t="str">
         <v>Legacy ID</v>
       </c>
-      <c r="I1" t="str">
-        <v>Active</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I1"/>
+      <c r="R1" t="str">
+        <v>Active*</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:R1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Checkpoint 39 – Contractor Recovery & NJ BRC UI Relocation
</commit_message>
<xml_diff>
--- a/public/SubTracker_Import_Template.xlsx
+++ b/public/SubTracker_Import_Template.xlsx
@@ -72,8 +72,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -405,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -432,9 +433,14 @@
         <v>Date columns accept Excel dates (MM/DD/YYYY).</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Taxpayer ID (FEIN) is optional and stored as text; enter 001234567 or 12-3456789. Do not append zeros.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -463,7 +469,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:S1"/>
+  <cols>
+    <col min="14" max="14" width="22" style="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -503,27 +512,30 @@
         <v>NJ BRC #</v>
       </c>
       <c r="M1" t="str">
+        <v>BRC Name Control</v>
+      </c>
+      <c r="N1" s="1" t="str">
+        <v>Taxpayer ID (FEIN)</v>
+      </c>
+      <c r="O1" t="str">
         <v>Sage ERP ID</v>
       </c>
-      <c r="N1" t="str">
-        <v>BRC Name Control</v>
-      </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Notes</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>External ID</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Legacy ID</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>Active*</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Checkpoint - myCOI Insurance, Add Contractor and Multi-Source Project Ownership
Migration execution status is UNKNOWN. Required schema objects were found in the shared database even though this session did not apply the migration.

Local checkpoint only. No migration execution, push or deployment authorized.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/SubTracker_Import_Template.xlsx
+++ b/public/SubTracker_Import_Template.xlsx
@@ -8,10 +8,9 @@
     <sheet name="Contractors" sheetId="3" r:id="rId3"/>
     <sheet name="Project Assignments" sheetId="4" r:id="rId4"/>
     <sheet name="Compliance Records" sheetId="5" r:id="rId5"/>
-    <sheet name="Insurance" sheetId="6" r:id="rId6"/>
-    <sheet name="Tiered Subs" sheetId="7" r:id="rId7"/>
-    <sheet name="Follow-Ups" sheetId="8" r:id="rId8"/>
-    <sheet name="_Lists" sheetId="9" r:id="rId9"/>
+    <sheet name="Tiered Subs" sheetId="6" r:id="rId6"/>
+    <sheet name="Follow-Ups" sheetId="7" r:id="rId7"/>
+    <sheet name="_Lists" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -406,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -420,27 +419,37 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Supported worksheets: Projects, Contractors, Project Assignments, Compliance Records, Insurance, Tiered Subs, Follow-Ups.</v>
+        <v>Supported worksheets: Projects, Contractors, Project Assignments, Compliance Records, Tiered Subs, Follow-Ups.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Yes/No columns accept Yes or No.</v>
+        <v>Manual Insurance and Certificate Of Insurance tracking are retired. Use the reviewed myCOI workflow for insurance.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Date columns accept Excel dates (MM/DD/YYYY).</v>
+        <v>Project Assignments controls MANUAL ownership only; it cannot remove MYCOI ownership.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Yes/No columns accept Yes or No.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Date columns accept Excel dates (MM/DD/YYYY).</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
         <v>Taxpayer ID (FEIN) is optional and stored as text; enter 001234567 or 12-3456789. Do not append zeros.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -613,37 +622,6 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Company Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>COI On File</v>
-      </c>
-      <c r="C1" t="str">
-        <v>General Liability On File</v>
-      </c>
-      <c r="D1" t="str">
-        <v>General Liability Expiration Date</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Workers Comp On File</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Workers Comp Expiration Date</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D1"/>
   <sheetData>
     <row r="1">
@@ -667,7 +645,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G1"/>
   <sheetData>
@@ -701,7 +679,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D7"/>
   <sheetData>

</xml_diff>